<commit_message>
Removed Output class and moved capabilities to Session + structure overhaul
</commit_message>
<xml_diff>
--- a/data/default/DemandAndConversions.xlsx
+++ b/data/default/DemandAndConversions.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Trade" sheetId="4" r:id="rId3"/>
     <sheet name="references" sheetId="5" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913" iterate="1"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1620" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1622" uniqueCount="358">
   <si>
     <t>parameter</t>
   </si>
@@ -1114,6 +1114,12 @@
   </si>
   <si>
     <t>for 2019</t>
+  </si>
+  <si>
+    <t>temp add 303000</t>
+  </si>
+  <si>
+    <t>temp add 246000</t>
   </si>
 </sst>
 </file>
@@ -1563,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N386"/>
+  <dimension ref="A1:R386"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.42578125" customWidth="1"/>
@@ -3295,7 +3301,7 @@
       <c r="M96" s="3"/>
       <c r="N96" s="3"/>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>295</v>
       </c>
@@ -3321,7 +3327,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>296</v>
       </c>
@@ -3335,7 +3341,8 @@
         <v>300</v>
       </c>
       <c r="K98" s="33">
-        <v>304650.40000000002</v>
+        <f>304650.4+303000</f>
+        <v>607650.4</v>
       </c>
       <c r="L98" t="s">
         <v>196</v>
@@ -3346,8 +3353,11 @@
       <c r="N98" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="R98" s="6" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>297</v>
       </c>
@@ -3373,7 +3383,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>298</v>
       </c>
@@ -3387,7 +3397,8 @@
         <v>300</v>
       </c>
       <c r="K100" s="33">
-        <v>177249.6</v>
+        <f>177249.6+246000</f>
+        <v>423249.6</v>
       </c>
       <c r="L100" t="s">
         <v>196</v>
@@ -3398,8 +3409,11 @@
       <c r="N100" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="R100" s="6" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="101" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>208</v>
       </c>
@@ -3425,7 +3439,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>101</v>
       </c>
@@ -3451,7 +3465,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>34</v>
       </c>
@@ -3469,7 +3483,7 @@
       <c r="M104" s="3"/>
       <c r="N104" s="3"/>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B105" t="s">
         <v>26</v>
       </c>
@@ -3486,7 +3500,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B106" t="s">
         <v>26</v>
       </c>
@@ -3503,7 +3517,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B107" t="s">
         <v>26</v>
       </c>
@@ -3523,7 +3537,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
         <v>103</v>
       </c>
@@ -3540,7 +3554,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B109" t="s">
         <v>103</v>
       </c>
@@ -3557,7 +3571,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B110" t="s">
         <v>103</v>
       </c>
@@ -3577,7 +3591,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
         <v>108</v>
       </c>
@@ -3594,7 +3608,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B112" t="s">
         <v>108</v>
       </c>

</xml_diff>

<commit_message>
Adjusted factors CW->retail weight to align with JBV factors
</commit_message>
<xml_diff>
--- a/data/default/DemandAndConversions.xlsx
+++ b/data/default/DemandAndConversions.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2515" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2515" uniqueCount="480">
   <si>
     <t>parameter</t>
   </si>
@@ -1097,12 +1097,6 @@
     <t>Unprocessed commodity</t>
   </si>
   <si>
-    <t>adjusted from 73% to match slaughter statistics</t>
-  </si>
-  <si>
-    <t>adjusted from 71% to match slaughter statistics</t>
-  </si>
-  <si>
     <t>population_region</t>
   </si>
   <si>
@@ -1433,15 +1427,9 @@
     <t>Incl. absorbed water. (1/0.78)=carcass weight--&gt;live weight</t>
   </si>
   <si>
-    <t>adjusted to match slaughter statistics. &lt;92% in ref.</t>
-  </si>
-  <si>
     <t xml:space="preserve">FAO 1992 / https://doi.org/10.3382/ps.0592243 </t>
   </si>
   <si>
-    <t>chanaged from 66% to match slaughter statistics</t>
-  </si>
-  <si>
     <t>assumed same as for bioethanol</t>
   </si>
   <si>
@@ -1511,7 +1499,13 @@
     <t>Avg. 2016-2020. (imp-exp)/consumption</t>
   </si>
   <si>
-    <t>Avg.2016-2020. Based on "totalkonsumtion" adjusted for assumed CW to retail weight factor and losses</t>
+    <t>JBV. Konsumtion animalieprodukter. Priser och marknads­information för livsmedel. https://jordbruksverket.se/mat-och-drycker/handel-och-marknad/priser-och-marknadsinformation-for-livsmedel</t>
+  </si>
+  <si>
+    <t>Retail weight</t>
+  </si>
+  <si>
+    <t>Avg.2016-2020. Based on "totalkonsumtion" adjusted with JBV factors for CW --&gt; retail weight</t>
   </si>
 </sst>
 </file>
@@ -2235,13 +2229,13 @@
         <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>26</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>55</v>
@@ -2308,7 +2302,7 @@
         <v>6</v>
       </c>
       <c r="O3" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="P3" t="s">
         <v>7</v>
@@ -2316,19 +2310,19 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="L4" t="s">
+        <v>343</v>
+      </c>
+      <c r="M4" s="30" t="s">
+        <v>347</v>
+      </c>
+      <c r="N4" t="s">
+        <v>344</v>
+      </c>
+      <c r="O4" t="s">
         <v>345</v>
       </c>
-      <c r="M4" s="30" t="s">
-        <v>349</v>
-      </c>
-      <c r="N4" t="s">
+      <c r="P4" t="s">
         <v>346</v>
-      </c>
-      <c r="O4" t="s">
-        <v>347</v>
-      </c>
-      <c r="P4" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -2635,7 +2629,7 @@
     </row>
     <row r="21" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B21" s="17" t="s">
         <v>25</v>
@@ -2790,7 +2784,7 @@
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B29" s="17" t="s">
         <v>105</v>
@@ -3331,7 +3325,7 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="17" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B59" s="17" t="s">
         <v>79</v>
@@ -3386,17 +3380,17 @@
         <v>17</v>
       </c>
       <c r="M61" s="22">
-        <f>31.8*1000/365.25 * 0.73 * (1-M188/100) * (1-M187/100) * (1-M186/100)</f>
-        <v>53.759619942505125</v>
+        <f>31.8*1000/365.25 * 0.78 * (1-M188/100) * (1-M187/100) * (1-M186/100)</f>
+        <v>57.44178569199179</v>
       </c>
       <c r="N61" t="s">
         <v>18</v>
       </c>
       <c r="O61" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="P61" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
@@ -3410,17 +3404,17 @@
         <v>17</v>
       </c>
       <c r="M62" s="22">
-        <f>24.5*1000/365.25 * 0.71 * (1-M188/100) * (1-M187/100) * (1-M186/100)</f>
-        <v>40.283819630390141</v>
+        <f>24.5*1000/365.25 * 0.7 * (1-M188/100) * (1-M187/100) * (1-M186/100)</f>
+        <v>39.716441889117036</v>
       </c>
       <c r="N62" t="s">
         <v>18</v>
       </c>
       <c r="O62" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="P62" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
@@ -3434,17 +3428,17 @@
         <v>17</v>
       </c>
       <c r="M63" s="29">
-        <f>1.8*1000/365.25 * 0.66 * (1-M188/100) * (1-M187/100) * (1-M186/100)</f>
-        <v>2.7512030882956875</v>
+        <f>1.8*1000/365.25 * 0.88 * (1-M188/100) * (1-M187/100) * (1-M186/100)</f>
+        <v>3.6682707843942506</v>
       </c>
       <c r="N63" t="s">
         <v>18</v>
       </c>
       <c r="O63" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="P63" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
@@ -3458,25 +3452,25 @@
         <v>17</v>
       </c>
       <c r="M64" s="22">
-        <f>22.7*1000/365.25 * 0.87 * (1-M188/100) * (1-M187/100) * (1-M186/100)</f>
-        <v>45.735277601642707</v>
+        <f>22.7*1000/365.25 * 0.88 * (1-M188/100) * (1-M187/100) * (1-M186/100)</f>
+        <v>46.260970447638599</v>
       </c>
       <c r="N64" t="s">
         <v>18</v>
       </c>
       <c r="O64" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="P64" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>428</v>
+      </c>
+      <c r="B65" t="s">
         <v>430</v>
-      </c>
-      <c r="B65" t="s">
-        <v>432</v>
       </c>
       <c r="L65" t="s">
         <v>17</v>
@@ -3488,15 +3482,15 @@
         <v>18</v>
       </c>
       <c r="O65" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B66" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="L66" t="s">
         <v>17</v>
@@ -3551,7 +3545,7 @@
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="17" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B69" s="17" t="s">
         <v>307</v>
@@ -3575,7 +3569,7 @@
         <v>18</v>
       </c>
       <c r="O69" s="17" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
@@ -3688,7 +3682,7 @@
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="17" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B76" s="17" t="s">
         <v>196</v>
@@ -3715,7 +3709,7 @@
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="17" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B77" s="17" t="s">
         <v>196</v>
@@ -3779,10 +3773,10 @@
     </row>
     <row r="80" spans="1:16" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="57" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B80" s="57" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C80" s="57"/>
       <c r="D80" s="58"/>
@@ -3807,10 +3801,10 @@
     </row>
     <row r="81" spans="1:16" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="57" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B81" s="57" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C81" s="57"/>
       <c r="D81" s="58"/>
@@ -3835,7 +3829,7 @@
     </row>
     <row r="82" spans="1:16" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="52" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B82" s="54"/>
       <c r="C82" s="54"/>
@@ -3855,10 +3849,10 @@
     </row>
     <row r="83" spans="1:16" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="57" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B83" s="57" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C83" s="57"/>
       <c r="D83" s="58"/>
@@ -3924,7 +3918,7 @@
     </row>
     <row r="86" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B86" s="17" t="s">
         <v>116</v>
@@ -3948,7 +3942,7 @@
         <v>18</v>
       </c>
       <c r="O86" s="17" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="87" spans="1:16" x14ac:dyDescent="0.25">
@@ -4243,10 +4237,10 @@
     </row>
     <row r="102" spans="1:16" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="57" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B102" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C102" s="57"/>
       <c r="D102" s="58"/>
@@ -4270,10 +4264,10 @@
     </row>
     <row r="103" spans="1:16" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="57" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B103" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C103" s="57"/>
       <c r="D103" s="58"/>
@@ -4294,15 +4288,15 @@
         <v>18</v>
       </c>
       <c r="O103" s="57" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="104" spans="1:16" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="57" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B104" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C104" s="57"/>
       <c r="D104" s="57"/>
@@ -4326,10 +4320,10 @@
     </row>
     <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A105" s="57" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B105" s="57" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C105" s="57"/>
       <c r="D105" s="57"/>
@@ -4353,10 +4347,10 @@
     </row>
     <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106" s="57" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B106" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C106" s="57"/>
       <c r="D106" s="58"/>
@@ -4381,10 +4375,10 @@
     </row>
     <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107" s="57" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B107" s="57" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C107" s="57"/>
       <c r="D107" s="58"/>
@@ -4409,10 +4403,10 @@
     </row>
     <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A108" s="57" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B108" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C108" s="57"/>
       <c r="D108" s="57"/>
@@ -4437,10 +4431,10 @@
     </row>
     <row r="109" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A109" s="57" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B109" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C109" s="57"/>
       <c r="D109" s="58"/>
@@ -4465,10 +4459,10 @@
     </row>
     <row r="110" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A110" s="57" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B110" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C110" s="57"/>
       <c r="D110" s="58"/>
@@ -4493,10 +4487,10 @@
     </row>
     <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A111" s="57" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B111" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C111" s="57"/>
       <c r="D111" s="58"/>
@@ -4521,10 +4515,10 @@
     </row>
     <row r="112" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A112" s="57" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B112" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C112" s="57"/>
       <c r="D112" s="58"/>
@@ -4549,10 +4543,10 @@
     </row>
     <row r="113" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A113" s="57" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B113" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C113" s="57"/>
       <c r="D113" s="58"/>
@@ -4577,10 +4571,10 @@
     </row>
     <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114" s="57" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B114" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C114" s="57"/>
       <c r="D114" s="17"/>
@@ -4673,7 +4667,7 @@
     </row>
     <row r="119" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A119" s="17" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B119" s="17" t="s">
         <v>189</v>
@@ -4699,7 +4693,7 @@
         <v>179</v>
       </c>
       <c r="O119" s="17" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="P119" s="7"/>
     </row>
@@ -4815,7 +4809,7 @@
     </row>
     <row r="129" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A129" s="17" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B129" t="s">
         <v>189</v>
@@ -4830,7 +4824,7 @@
         <v>1000</v>
       </c>
       <c r="N129" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="O129" s="6"/>
       <c r="P129" s="9"/>
@@ -4878,7 +4872,7 @@
         <v>179</v>
       </c>
       <c r="O132" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="P132" t="s">
         <v>281</v>
@@ -4905,7 +4899,7 @@
         <v>179</v>
       </c>
       <c r="O133" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="P133" t="s">
         <v>281</v>
@@ -4934,7 +4928,7 @@
         <v>179</v>
       </c>
       <c r="O134" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="P134" t="s">
         <v>281</v>
@@ -4960,7 +4954,7 @@
         <v>179</v>
       </c>
       <c r="O135" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="P135" t="s">
         <v>281</v>
@@ -4989,7 +4983,7 @@
         <v>179</v>
       </c>
       <c r="O136" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="P136" t="s">
         <v>281</v>
@@ -5107,7 +5101,7 @@
         <v>179</v>
       </c>
       <c r="O140" s="17" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="P140">
         <v>20000</v>
@@ -5260,7 +5254,7 @@
     </row>
     <row r="146" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A146" s="17" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B146" s="17" t="s">
         <v>79</v>
@@ -5289,7 +5283,7 @@
     </row>
     <row r="147" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A147" s="17" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B147" s="17" t="s">
         <v>79</v>
@@ -5344,7 +5338,7 @@
         <v>179</v>
       </c>
       <c r="O148" s="17" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="149" spans="1:15" x14ac:dyDescent="0.25">
@@ -5378,10 +5372,10 @@
     </row>
     <row r="150" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A150" s="57" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B150" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C150" s="17"/>
       <c r="D150" s="17"/>
@@ -5407,10 +5401,10 @@
     </row>
     <row r="151" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A151" s="57" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B151" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C151" s="17"/>
       <c r="D151" s="17"/>
@@ -5436,10 +5430,10 @@
     </row>
     <row r="152" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A152" s="57" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B152" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C152" s="17"/>
       <c r="D152" s="17"/>
@@ -5465,10 +5459,10 @@
     </row>
     <row r="153" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A153" s="57" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B153" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C153" s="17"/>
       <c r="D153" s="17"/>
@@ -5494,10 +5488,10 @@
     </row>
     <row r="154" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A154" s="57" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B154" s="57" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C154" s="17"/>
       <c r="D154" s="17"/>
@@ -5523,10 +5517,10 @@
     </row>
     <row r="155" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A155" s="57" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B155" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C155" s="17"/>
       <c r="D155" s="17"/>
@@ -5552,10 +5546,10 @@
     </row>
     <row r="156" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A156" s="57" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B156" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C156" s="17"/>
       <c r="D156" s="17"/>
@@ -5581,10 +5575,10 @@
     </row>
     <row r="157" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A157" s="17" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B157" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C157" s="17"/>
       <c r="D157" s="17"/>
@@ -5610,10 +5604,10 @@
     </row>
     <row r="158" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A158" s="17" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B158" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C158" s="17"/>
       <c r="D158" s="17"/>
@@ -5639,10 +5633,10 @@
     </row>
     <row r="159" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A159" s="17" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B159" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C159" s="17"/>
       <c r="D159" s="17"/>
@@ -5668,10 +5662,10 @@
     </row>
     <row r="160" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A160" s="17" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B160" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C160" s="17"/>
       <c r="D160" s="17"/>
@@ -5697,7 +5691,7 @@
     </row>
     <row r="162" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A162" s="61" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
@@ -5717,33 +5711,33 @@
     </row>
     <row r="163" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A163" s="62" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="164" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A164" s="62" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="165" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A165" s="62" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="166" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A166" s="62" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="167" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A167" s="57" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C167" t="s">
         <v>191</v>
       </c>
       <c r="L167" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="M167">
         <v>50</v>
@@ -5752,18 +5746,18 @@
         <v>37</v>
       </c>
       <c r="O167" s="6" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="168" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A168" s="57" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C168" t="s">
         <v>115</v>
       </c>
       <c r="L168" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="M168">
         <v>50</v>
@@ -5809,7 +5803,7 @@
         <v>37</v>
       </c>
       <c r="P171" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="172" spans="1:16" x14ac:dyDescent="0.25">
@@ -5829,7 +5823,7 @@
         <v>37</v>
       </c>
       <c r="P172" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="173" spans="1:16" x14ac:dyDescent="0.25">
@@ -5850,7 +5844,7 @@
       </c>
       <c r="O173" s="6"/>
       <c r="P173" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="174" spans="1:16" x14ac:dyDescent="0.25">
@@ -5870,7 +5864,7 @@
         <v>37</v>
       </c>
       <c r="P174" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="175" spans="1:16" x14ac:dyDescent="0.25">
@@ -5890,7 +5884,7 @@
         <v>37</v>
       </c>
       <c r="P175" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="176" spans="1:16" x14ac:dyDescent="0.25">
@@ -5911,7 +5905,7 @@
       </c>
       <c r="O176" s="6"/>
       <c r="P176" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="177" spans="2:16" x14ac:dyDescent="0.25">
@@ -5931,7 +5925,7 @@
         <v>37</v>
       </c>
       <c r="P177" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="178" spans="2:16" x14ac:dyDescent="0.25">
@@ -5951,7 +5945,7 @@
         <v>37</v>
       </c>
       <c r="P178" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="179" spans="2:16" x14ac:dyDescent="0.25">
@@ -5972,7 +5966,7 @@
       </c>
       <c r="O179" s="6"/>
       <c r="P179" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="180" spans="2:16" x14ac:dyDescent="0.25">
@@ -5992,7 +5986,7 @@
         <v>37</v>
       </c>
       <c r="P180" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="181" spans="2:16" x14ac:dyDescent="0.25">
@@ -6012,7 +6006,7 @@
         <v>37</v>
       </c>
       <c r="P181" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="182" spans="2:16" x14ac:dyDescent="0.25">
@@ -6033,7 +6027,7 @@
       </c>
       <c r="O182" s="6"/>
       <c r="P182" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="183" spans="2:16" x14ac:dyDescent="0.25">
@@ -6053,7 +6047,7 @@
         <v>37</v>
       </c>
       <c r="P183" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="184" spans="2:16" x14ac:dyDescent="0.25">
@@ -6074,7 +6068,7 @@
         <v>37</v>
       </c>
       <c r="P184" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="185" spans="2:16" x14ac:dyDescent="0.25">
@@ -6095,7 +6089,7 @@
       </c>
       <c r="O185" s="6"/>
       <c r="P185" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="186" spans="2:16" x14ac:dyDescent="0.25">
@@ -6115,7 +6109,7 @@
         <v>37</v>
       </c>
       <c r="P186" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="187" spans="2:16" x14ac:dyDescent="0.25">
@@ -6135,7 +6129,7 @@
         <v>37</v>
       </c>
       <c r="P187" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="188" spans="2:16" x14ac:dyDescent="0.25">
@@ -6155,15 +6149,15 @@
         <v>37</v>
       </c>
       <c r="O188" s="17" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="P188" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="189" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B189" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="K189" t="s">
         <v>49</v>
@@ -6179,12 +6173,12 @@
         <v>37</v>
       </c>
       <c r="O189" s="17" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="190" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B190" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="K190" t="s">
         <v>50</v>
@@ -6203,7 +6197,7 @@
     </row>
     <row r="191" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B191" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="K191" t="s">
         <v>51</v>
@@ -6237,7 +6231,7 @@
         <v>37</v>
       </c>
       <c r="P192" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="193" spans="1:16" x14ac:dyDescent="0.25">
@@ -6257,7 +6251,7 @@
         <v>37</v>
       </c>
       <c r="P193" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="194" spans="1:16" x14ac:dyDescent="0.25">
@@ -6278,7 +6272,7 @@
       </c>
       <c r="O194" s="6"/>
       <c r="P194" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="195" spans="1:16" x14ac:dyDescent="0.25">
@@ -6298,7 +6292,7 @@
         <v>37</v>
       </c>
       <c r="P195" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="196" spans="1:16" x14ac:dyDescent="0.25">
@@ -6318,7 +6312,7 @@
         <v>37</v>
       </c>
       <c r="P196" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="197" spans="1:16" x14ac:dyDescent="0.25">
@@ -6339,7 +6333,7 @@
       </c>
       <c r="O197" s="6"/>
       <c r="P197" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="198" spans="1:16" x14ac:dyDescent="0.25">
@@ -6359,7 +6353,7 @@
         <v>37</v>
       </c>
       <c r="P198" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="199" spans="1:16" x14ac:dyDescent="0.25">
@@ -6379,7 +6373,7 @@
         <v>37</v>
       </c>
       <c r="P199" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="200" spans="1:16" x14ac:dyDescent="0.25">
@@ -6400,7 +6394,7 @@
       </c>
       <c r="O200" s="6"/>
       <c r="P200" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="201" spans="1:16" x14ac:dyDescent="0.25">
@@ -6420,7 +6414,7 @@
         <v>37</v>
       </c>
       <c r="P201" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="202" spans="1:16" x14ac:dyDescent="0.25">
@@ -6440,7 +6434,7 @@
         <v>37</v>
       </c>
       <c r="P202" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="203" spans="1:16" x14ac:dyDescent="0.25">
@@ -6461,7 +6455,7 @@
       </c>
       <c r="O203" s="6"/>
       <c r="P203" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="204" spans="1:16" x14ac:dyDescent="0.25">
@@ -6481,7 +6475,7 @@
         <v>37</v>
       </c>
       <c r="P204" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="205" spans="1:16" x14ac:dyDescent="0.25">
@@ -6501,7 +6495,7 @@
         <v>37</v>
       </c>
       <c r="P205" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="206" spans="1:16" x14ac:dyDescent="0.25">
@@ -6522,13 +6516,13 @@
       </c>
       <c r="O206" s="6"/>
       <c r="P206" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="207" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A207" s="7"/>
       <c r="B207" s="17" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C207" s="17"/>
       <c r="D207" s="17"/>
@@ -6552,13 +6546,13 @@
         <v>37</v>
       </c>
       <c r="O207" s="17" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="208" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A208" s="7"/>
       <c r="B208" s="17" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C208" s="17"/>
       <c r="D208" s="17"/>
@@ -6586,7 +6580,7 @@
     <row r="209" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A209" s="7"/>
       <c r="B209" s="17" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C209" s="17"/>
       <c r="D209" s="17"/>
@@ -6614,7 +6608,7 @@
     <row r="210" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A210" s="7"/>
       <c r="B210" s="57" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C210" s="57"/>
       <c r="D210" s="17"/>
@@ -6638,13 +6632,13 @@
         <v>37</v>
       </c>
       <c r="O210" s="17" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="211" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A211" s="7"/>
       <c r="B211" s="57" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C211" s="57"/>
       <c r="D211" s="17"/>
@@ -6671,7 +6665,7 @@
     </row>
     <row r="212" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B212" s="57" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C212" s="57"/>
       <c r="D212" s="17"/>
@@ -6698,7 +6692,7 @@
     </row>
     <row r="213" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B213" s="57" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C213" s="57"/>
       <c r="D213" s="17"/>
@@ -6722,12 +6716,12 @@
       </c>
       <c r="O213" s="6"/>
       <c r="P213" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="214" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B214" s="57" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C214" s="57"/>
       <c r="D214" s="17"/>
@@ -6751,12 +6745,12 @@
       </c>
       <c r="O214" s="6"/>
       <c r="P214" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="215" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B215" s="57" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C215" s="57"/>
       <c r="D215" s="17"/>
@@ -6780,12 +6774,12 @@
       </c>
       <c r="O215" s="6"/>
       <c r="P215" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="216" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B216" s="57" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C216" s="57"/>
       <c r="D216" s="17"/>
@@ -6809,12 +6803,12 @@
       </c>
       <c r="O216" s="6"/>
       <c r="P216" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="217" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B217" s="57" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C217" s="57"/>
       <c r="D217" s="17"/>
@@ -6838,12 +6832,12 @@
       </c>
       <c r="O217" s="6"/>
       <c r="P217" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="218" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B218" s="57" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C218" s="57"/>
       <c r="D218" s="17"/>
@@ -6867,7 +6861,7 @@
       </c>
       <c r="O218" s="6"/>
       <c r="P218" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="219" spans="1:16" x14ac:dyDescent="0.25">
@@ -7139,7 +7133,7 @@
     </row>
     <row r="236" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A236" s="17" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="L236" s="17" t="s">
         <v>39</v>
@@ -7406,7 +7400,7 @@
     </row>
     <row r="253" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A253" s="17" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B253" s="17"/>
       <c r="C253" s="17"/>
@@ -7428,7 +7422,7 @@
         <v>37</v>
       </c>
       <c r="O253" s="17" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="254" spans="1:16" x14ac:dyDescent="0.25">
@@ -7519,7 +7513,7 @@
         <v>37</v>
       </c>
       <c r="O259" s="6" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
     </row>
     <row r="260" spans="1:16" x14ac:dyDescent="0.25">
@@ -7536,7 +7530,7 @@
         <v>37</v>
       </c>
       <c r="O260" s="6" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
     </row>
     <row r="261" spans="1:16" x14ac:dyDescent="0.25">
@@ -7731,7 +7725,7 @@
     </row>
     <row r="273" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A273" s="17" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="L273" s="17" t="s">
         <v>39</v>
@@ -7743,7 +7737,7 @@
         <v>37</v>
       </c>
       <c r="O273" s="17" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="274" spans="1:16" x14ac:dyDescent="0.25">
@@ -7780,10 +7774,10 @@
         <v>37</v>
       </c>
       <c r="O275" s="17" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="P275" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
     </row>
     <row r="276" spans="1:16" x14ac:dyDescent="0.25">
@@ -7800,10 +7794,10 @@
         <v>37</v>
       </c>
       <c r="O276" s="17" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="P276" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
     </row>
     <row r="277" spans="1:16" x14ac:dyDescent="0.25">
@@ -7820,10 +7814,10 @@
         <v>37</v>
       </c>
       <c r="O277" s="17" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="P277" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
     </row>
     <row r="278" spans="1:16" x14ac:dyDescent="0.25">
@@ -7840,15 +7834,15 @@
         <v>37</v>
       </c>
       <c r="O278" s="17" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="P278" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
     </row>
     <row r="279" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="L279" t="s">
         <v>39</v>
@@ -7860,12 +7854,12 @@
         <v>37</v>
       </c>
       <c r="O279" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="280" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="L280" t="s">
         <v>39</v>
@@ -7914,7 +7908,7 @@
     </row>
     <row r="283" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A283" s="17" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B283" s="17"/>
       <c r="C283" s="17"/>
@@ -8044,7 +8038,7 @@
     </row>
     <row r="290" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A290" s="17" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B290" s="19"/>
       <c r="C290" s="19"/>
@@ -8066,13 +8060,13 @@
         <v>37</v>
       </c>
       <c r="O290" s="19" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="P290" s="19"/>
     </row>
     <row r="291" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A291" s="17" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B291" s="19"/>
       <c r="C291" s="19"/>
@@ -8094,7 +8088,7 @@
         <v>37</v>
       </c>
       <c r="O291" s="19" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="P291" s="19"/>
     </row>
@@ -8120,7 +8114,7 @@
     </row>
     <row r="293" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A293" s="17" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B293" s="19"/>
       <c r="C293" s="19"/>
@@ -8142,13 +8136,13 @@
         <v>37</v>
       </c>
       <c r="O293" s="49" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="P293" s="49"/>
     </row>
     <row r="294" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A294" s="17" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B294" s="19"/>
       <c r="C294" s="19"/>
@@ -8170,13 +8164,13 @@
         <v>37</v>
       </c>
       <c r="O294" s="49" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="P294" s="49"/>
     </row>
     <row r="295" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A295" s="52" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B295" s="53"/>
       <c r="C295" s="53"/>
@@ -8196,7 +8190,7 @@
     </row>
     <row r="296" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A296" s="17" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B296" s="19"/>
       <c r="C296" s="19"/>
@@ -8218,7 +8212,7 @@
         <v>37</v>
       </c>
       <c r="O296" s="49" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="P296" s="49"/>
     </row>
@@ -8259,7 +8253,7 @@
     </row>
     <row r="299" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A299" s="17" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="L299" s="17" t="s">
         <v>39</v>
@@ -8271,7 +8265,7 @@
         <v>37</v>
       </c>
       <c r="O299" s="56" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="300" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
@@ -8465,10 +8459,10 @@
     </row>
     <row r="311" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A311" s="57" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B311" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C311" s="57"/>
       <c r="D311" s="58"/>
@@ -8489,15 +8483,15 @@
         <v>37</v>
       </c>
       <c r="O311" s="57" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="312" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A312" s="57" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B312" s="57" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C312" s="57"/>
       <c r="D312" s="58"/>
@@ -8518,15 +8512,15 @@
         <v>37</v>
       </c>
       <c r="O312" s="57" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="313" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A313" s="57" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B313" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C313" s="57"/>
       <c r="D313" s="57"/>
@@ -8547,16 +8541,16 @@
         <v>37</v>
       </c>
       <c r="O313" s="57" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="P313" s="57"/>
     </row>
     <row r="314" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A314" s="17" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B314" s="17" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="L314" s="17" t="s">
         <v>39</v>
@@ -8568,15 +8562,15 @@
         <v>37</v>
       </c>
       <c r="O314" s="57" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="315" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A315" s="57" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B315" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C315" s="57"/>
       <c r="D315" s="58"/>
@@ -8597,15 +8591,15 @@
         <v>37</v>
       </c>
       <c r="O315" s="57" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="316" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A316" s="57" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B316" s="57" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C316" s="57"/>
       <c r="D316" s="58"/>
@@ -8626,15 +8620,15 @@
         <v>37</v>
       </c>
       <c r="O316" s="57" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="317" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A317" s="57" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B317" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C317" s="57"/>
       <c r="D317" s="58"/>
@@ -8655,15 +8649,15 @@
         <v>37</v>
       </c>
       <c r="O317" s="57" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="318" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A318" s="57" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B318" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C318" s="57"/>
       <c r="D318" s="58"/>
@@ -8684,15 +8678,15 @@
         <v>37</v>
       </c>
       <c r="O318" s="57" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="319" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A319" s="57" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B319" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C319" s="57"/>
       <c r="D319" s="58"/>
@@ -8713,15 +8707,15 @@
         <v>37</v>
       </c>
       <c r="O319" s="57" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="320" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A320" s="57" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B320" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C320" s="57"/>
       <c r="D320" s="58"/>
@@ -8742,15 +8736,15 @@
         <v>37</v>
       </c>
       <c r="O320" s="57" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="321" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A321" s="57" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B321" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C321" s="57"/>
       <c r="D321" s="58"/>
@@ -8771,15 +8765,15 @@
         <v>37</v>
       </c>
       <c r="O321" s="57" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="322" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A322" s="57" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B322" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C322" s="57"/>
       <c r="D322" s="58"/>
@@ -8800,15 +8794,15 @@
         <v>37</v>
       </c>
       <c r="O322" s="57" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="323" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A323" s="57" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B323" s="57" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C323" s="57"/>
       <c r="L323" s="57" t="s">
@@ -8821,7 +8815,7 @@
         <v>37</v>
       </c>
       <c r="O323" s="57" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="325" spans="1:16" x14ac:dyDescent="0.25">
@@ -9134,7 +9128,7 @@
     </row>
     <row r="339" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A339" s="17" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="I339" s="17" t="s">
         <v>85</v>
@@ -9152,7 +9146,7 @@
         <v>37</v>
       </c>
       <c r="O339" s="17" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="340" spans="1:16" x14ac:dyDescent="0.25">
@@ -9309,7 +9303,7 @@
     </row>
     <row r="347" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A347" s="17" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="I347" s="17" t="s">
         <v>85</v>
@@ -9327,7 +9321,7 @@
         <v>37</v>
       </c>
       <c r="O347" s="17" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="P347" s="17" t="s">
         <v>156</v>
@@ -9733,7 +9727,7 @@
     </row>
     <row r="365" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="I365" t="s">
         <v>85</v>
@@ -9752,12 +9746,12 @@
         <v>37</v>
       </c>
       <c r="O365" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="366" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="I366" t="s">
         <v>85</v>
@@ -9776,7 +9770,7 @@
         <v>37</v>
       </c>
       <c r="O366" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="367" spans="1:16" x14ac:dyDescent="0.25">
@@ -9827,7 +9821,7 @@
     </row>
     <row r="369" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A369" s="17" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="I369" s="17" t="s">
         <v>85</v>
@@ -9910,7 +9904,7 @@
     </row>
     <row r="373" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A373" s="17" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="I373" s="17" t="s">
         <v>85</v>
@@ -9928,12 +9922,12 @@
         <v>37</v>
       </c>
       <c r="O373" s="17" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="374" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A374" s="17" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="I374" s="17" t="s">
         <v>85</v>
@@ -9951,12 +9945,12 @@
         <v>37</v>
       </c>
       <c r="O374" s="17" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="375" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A375" s="52" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B375" s="54"/>
       <c r="C375" s="54"/>
@@ -9976,7 +9970,7 @@
     </row>
     <row r="376" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A376" s="17" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="I376" s="17" t="s">
         <v>85</v>
@@ -9994,7 +9988,7 @@
         <v>37</v>
       </c>
       <c r="O376" s="17" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="377" spans="1:16" x14ac:dyDescent="0.25">
@@ -10039,7 +10033,7 @@
     </row>
     <row r="379" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A379" s="57" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B379" s="57"/>
       <c r="C379" s="57"/>
@@ -10199,7 +10193,7 @@
     </row>
     <row r="386" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A386" s="57" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B386" s="57"/>
       <c r="C386" s="57"/>
@@ -10223,12 +10217,12 @@
         <v>37</v>
       </c>
       <c r="O386" s="57" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="387" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A387" s="57" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B387" s="57"/>
       <c r="C387" s="57"/>
@@ -10252,12 +10246,12 @@
         <v>37</v>
       </c>
       <c r="O387" s="57" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="388" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A388" s="17" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="J388" s="17" t="s">
         <v>42</v>
@@ -10272,7 +10266,7 @@
         <v>37</v>
       </c>
       <c r="O388" s="57" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="391" spans="1:16" x14ac:dyDescent="0.25">
@@ -10909,12 +10903,12 @@
     </row>
     <row r="414" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A414" s="48" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B414" s="68"/>
       <c r="C414" s="68"/>
       <c r="D414" s="69" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="E414" s="69"/>
       <c r="F414" s="68"/>
@@ -11171,10 +11165,10 @@
     </row>
     <row r="424" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A424" s="17" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D424" s="18" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="E424" s="18"/>
       <c r="L424" s="17" t="s">
@@ -11577,7 +11571,7 @@
       </c>
       <c r="R443" s="76"/>
       <c r="S443" s="77" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
     </row>
     <row r="444" spans="1:19" x14ac:dyDescent="0.25">
@@ -11600,7 +11594,7 @@
       <c r="O444" s="5"/>
       <c r="P444" s="5"/>
       <c r="R444" s="72" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="S444" s="79">
         <v>4.2000000000000003E-2</v>
@@ -11608,7 +11602,7 @@
     </row>
     <row r="445" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A445" s="83" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="B445" s="83"/>
       <c r="C445" s="83"/>
@@ -11978,7 +11972,7 @@
     </row>
     <row r="455" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A455" s="83" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="B455" s="10"/>
       <c r="C455" s="10"/>
@@ -12223,7 +12217,7 @@
     </row>
     <row r="462" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A462" s="83" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="B462" s="10"/>
       <c r="C462" s="10"/>
@@ -12348,7 +12342,7 @@
     </row>
     <row r="466" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A466" s="10" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B466" s="8"/>
       <c r="C466" s="8"/>
@@ -12408,17 +12402,17 @@
       <c r="L468" t="s">
         <v>83</v>
       </c>
-      <c r="M468" s="11">
-        <v>73</v>
+      <c r="M468" s="18">
+        <v>78</v>
       </c>
       <c r="N468" s="8" t="s">
         <v>37</v>
       </c>
       <c r="O468" s="46" t="s">
-        <v>343</v>
-      </c>
-      <c r="P468" s="8" t="s">
-        <v>89</v>
+        <v>478</v>
+      </c>
+      <c r="P468" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="469" spans="1:19" x14ac:dyDescent="0.25">
@@ -12436,7 +12430,7 @@
         <v>54</v>
       </c>
       <c r="H469" s="8" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="I469" s="8"/>
       <c r="J469" s="8"/>
@@ -12473,7 +12467,7 @@
         <v>54</v>
       </c>
       <c r="H470" s="8" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="I470" s="8"/>
       <c r="J470" s="8"/>
@@ -12510,7 +12504,7 @@
         <v>54</v>
       </c>
       <c r="H471" s="8" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="I471" s="8"/>
       <c r="J471" s="8"/>
@@ -12547,7 +12541,7 @@
         <v>54</v>
       </c>
       <c r="H472" s="9" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="I472" s="8"/>
       <c r="J472" s="8"/>
@@ -12563,10 +12557,10 @@
         <v>37</v>
       </c>
       <c r="O472" s="9" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="P472" s="64" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="473" spans="1:19" x14ac:dyDescent="0.25">
@@ -12584,7 +12578,7 @@
         <v>54</v>
       </c>
       <c r="H473" s="8" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="I473" s="8"/>
       <c r="J473" s="8"/>
@@ -12624,17 +12618,17 @@
       <c r="L474" t="s">
         <v>83</v>
       </c>
-      <c r="M474" s="11">
-        <v>71</v>
+      <c r="M474" s="18">
+        <v>70</v>
       </c>
       <c r="N474" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="O474" s="9" t="s">
-        <v>344</v>
-      </c>
-      <c r="P474" s="8" t="s">
-        <v>89</v>
+      <c r="O474" s="46" t="s">
+        <v>478</v>
+      </c>
+      <c r="P474" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="475" spans="1:19" x14ac:dyDescent="0.25">
@@ -12652,7 +12646,7 @@
         <v>54</v>
       </c>
       <c r="H475" s="9" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="I475" s="8"/>
       <c r="J475" s="8"/>
@@ -12689,7 +12683,7 @@
         <v>54</v>
       </c>
       <c r="H476" s="8" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="I476" s="8"/>
       <c r="J476" s="8"/>
@@ -12726,7 +12720,7 @@
         <v>54</v>
       </c>
       <c r="H477" s="9" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="I477" s="8"/>
       <c r="J477" s="8"/>
@@ -12763,7 +12757,7 @@
         <v>54</v>
       </c>
       <c r="H478" s="9" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="I478" s="8"/>
       <c r="J478" s="8"/>
@@ -12779,10 +12773,10 @@
         <v>37</v>
       </c>
       <c r="O478" s="9" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="P478" s="64" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="479" spans="1:19" x14ac:dyDescent="0.25">
@@ -12800,7 +12794,7 @@
         <v>54</v>
       </c>
       <c r="H479" s="8" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="I479" s="8"/>
       <c r="J479" s="8"/>
@@ -12840,17 +12834,17 @@
       <c r="L480" t="s">
         <v>83</v>
       </c>
-      <c r="M480" s="11">
-        <v>66</v>
+      <c r="M480" s="18">
+        <v>88</v>
       </c>
       <c r="N480" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="O480" s="9" t="s">
-        <v>457</v>
-      </c>
-      <c r="P480" s="26" t="s">
-        <v>329</v>
+      <c r="O480" s="46" t="s">
+        <v>478</v>
+      </c>
+      <c r="P480" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="481" spans="1:16" x14ac:dyDescent="0.25">
@@ -12868,7 +12862,7 @@
         <v>54</v>
       </c>
       <c r="H481" s="9" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="I481" s="26"/>
       <c r="J481" s="26"/>
@@ -12905,7 +12899,7 @@
         <v>54</v>
       </c>
       <c r="H482" s="26" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="I482" s="8"/>
       <c r="J482" s="8"/>
@@ -12942,7 +12936,7 @@
         <v>54</v>
       </c>
       <c r="H483" s="9" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="I483" s="8"/>
       <c r="J483" s="8"/>
@@ -12958,7 +12952,7 @@
         <v>37</v>
       </c>
       <c r="O483" s="9" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="P483" s="26"/>
     </row>
@@ -12977,7 +12971,7 @@
         <v>54</v>
       </c>
       <c r="H484" s="26" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="I484" s="8"/>
       <c r="J484" s="8"/>
@@ -13020,17 +13014,17 @@
       <c r="L485" t="s">
         <v>83</v>
       </c>
-      <c r="M485" s="11">
-        <v>87</v>
+      <c r="M485" s="18">
+        <v>88</v>
       </c>
       <c r="N485" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="O485" s="9" t="s">
-        <v>455</v>
-      </c>
-      <c r="P485" s="8" t="s">
-        <v>89</v>
+      <c r="O485" s="46" t="s">
+        <v>478</v>
+      </c>
+      <c r="P485" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="486" spans="1:16" x14ac:dyDescent="0.25">
@@ -13048,7 +13042,7 @@
         <v>54</v>
       </c>
       <c r="H486" s="26" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="I486" s="8"/>
       <c r="J486" s="8"/>
@@ -13064,10 +13058,10 @@
         <v>37</v>
       </c>
       <c r="O486" s="9" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="P486" s="8" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="487" spans="1:16" x14ac:dyDescent="0.25">
@@ -13085,7 +13079,7 @@
         <v>54</v>
       </c>
       <c r="H487" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="L487" t="s">
         <v>84</v>
@@ -13099,7 +13093,7 @@
       </c>
       <c r="O487" s="9"/>
       <c r="P487" s="8" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="488" spans="1:16" x14ac:dyDescent="0.25">
@@ -13117,7 +13111,7 @@
         <v>54</v>
       </c>
       <c r="H488" s="9" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="I488" s="8"/>
       <c r="J488" s="8"/>
@@ -13134,7 +13128,7 @@
       </c>
       <c r="O488" s="9"/>
       <c r="P488" s="8" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="489" spans="1:16" x14ac:dyDescent="0.25">
@@ -13155,10 +13149,10 @@
     </row>
     <row r="490" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="H490" s="8" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="L490" t="s">
         <v>83</v>
@@ -13172,10 +13166,10 @@
     </row>
     <row r="491" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="H491" s="9" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="L491" t="s">
         <v>83</v>
@@ -13239,7 +13233,7 @@
     </row>
     <row r="494" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A494" s="6" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B494" s="10"/>
       <c r="C494" s="10"/>
@@ -13350,7 +13344,7 @@
       <c r="B500" s="19"/>
       <c r="C500" s="19"/>
       <c r="D500" s="19" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E500" s="19"/>
       <c r="F500" s="18"/>
@@ -13373,12 +13367,12 @@
     </row>
     <row r="501" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A501" s="17" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B501" s="19"/>
       <c r="C501" s="19"/>
       <c r="D501" s="19" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E501" s="19"/>
       <c r="F501" s="18"/>
@@ -13401,12 +13395,12 @@
     </row>
     <row r="502" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A502" s="17" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B502" s="19"/>
       <c r="C502" s="19"/>
       <c r="D502" s="19" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E502" s="19"/>
       <c r="F502" s="18"/>
@@ -13449,12 +13443,12 @@
     </row>
     <row r="504" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A504" s="48" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B504" s="68"/>
       <c r="C504" s="68"/>
       <c r="D504" s="68" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="E504" s="68"/>
       <c r="F504" s="69"/>
@@ -13477,18 +13471,18 @@
     </row>
     <row r="505" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A505" s="48" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B505" s="68"/>
       <c r="C505" s="68"/>
       <c r="D505" s="68" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="E505" s="68"/>
       <c r="F505" s="69"/>
       <c r="G505" s="69"/>
       <c r="H505" s="68" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="I505" s="68"/>
       <c r="J505" s="68"/>
@@ -13507,12 +13501,12 @@
     </row>
     <row r="506" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A506" s="48" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B506" s="68"/>
       <c r="C506" s="68"/>
       <c r="D506" s="68" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="E506" s="68"/>
       <c r="F506" s="69"/>
@@ -13535,18 +13529,18 @@
     </row>
     <row r="507" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A507" s="48" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B507" s="68"/>
       <c r="C507" s="68"/>
       <c r="D507" s="68" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="E507" s="68"/>
       <c r="F507" s="69"/>
       <c r="G507" s="69"/>
       <c r="H507" s="68" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="I507" s="68"/>
       <c r="J507" s="68"/>
@@ -13565,7 +13559,7 @@
     </row>
     <row r="508" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A508" s="52" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B508" s="53"/>
       <c r="C508" s="53"/>
@@ -13585,12 +13579,12 @@
     </row>
     <row r="509" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A509" s="48" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B509" s="68"/>
       <c r="C509" s="68"/>
       <c r="D509" s="68" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="E509" s="68"/>
       <c r="F509" s="69"/>
@@ -13731,7 +13725,7 @@
     </row>
     <row r="515" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A515" s="17" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D515" s="17" t="s">
         <v>117</v>
@@ -13752,7 +13746,7 @@
     </row>
     <row r="516" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A516" s="17" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D516" s="17" t="s">
         <v>117</v>
@@ -13776,7 +13770,7 @@
     </row>
     <row r="517" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A517" s="17" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D517" s="17" t="s">
         <v>117</v>
@@ -13797,7 +13791,7 @@
     </row>
     <row r="518" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A518" s="17" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D518" s="17" t="s">
         <v>117</v>
@@ -13824,7 +13818,7 @@
         <v>122</v>
       </c>
       <c r="D519" s="17" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="L519" s="17" t="s">
         <v>83</v>
@@ -13836,7 +13830,7 @@
         <v>37</v>
       </c>
       <c r="O519" s="17" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="P519" s="19"/>
     </row>
@@ -13845,10 +13839,10 @@
         <v>122</v>
       </c>
       <c r="D520" s="17" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="H520" s="17" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="L520" s="17" t="s">
         <v>84</v>
@@ -14284,7 +14278,7 @@
         <v>37</v>
       </c>
       <c r="O537" s="19" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="P537" s="10"/>
     </row>
@@ -14310,7 +14304,7 @@
     </row>
     <row r="539" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A539" s="57" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B539" s="57"/>
       <c r="C539" s="57"/>
@@ -14338,7 +14332,7 @@
     </row>
     <row r="540" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A540" s="57" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B540" s="57"/>
       <c r="C540" s="57"/>
@@ -14349,7 +14343,7 @@
       <c r="F540" s="58"/>
       <c r="G540" s="58"/>
       <c r="H540" s="57" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="I540" s="58"/>
       <c r="J540" s="57"/>
@@ -14365,13 +14359,13 @@
         <v>37</v>
       </c>
       <c r="O540" s="57" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="P540" s="19"/>
     </row>
     <row r="541" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A541" s="57" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B541" s="57"/>
       <c r="C541" s="57"/>
@@ -14395,13 +14389,13 @@
         <v>37</v>
       </c>
       <c r="O541" s="57" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="P541" s="19"/>
     </row>
     <row r="542" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A542" s="57" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B542" s="57"/>
       <c r="C542" s="57"/>
@@ -14412,7 +14406,7 @@
       <c r="F542" s="57"/>
       <c r="G542" s="57"/>
       <c r="H542" s="57" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="I542" s="57"/>
       <c r="J542" s="57"/>
@@ -14432,7 +14426,7 @@
     </row>
     <row r="543" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A543" s="57" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B543" s="57"/>
       <c r="C543" s="57"/>
@@ -14443,7 +14437,7 @@
       <c r="F543" s="57"/>
       <c r="G543" s="57"/>
       <c r="H543" s="57" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="I543" s="57"/>
       <c r="J543" s="57"/>
@@ -14463,7 +14457,7 @@
     </row>
     <row r="544" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A544" s="57" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B544" s="57"/>
       <c r="C544" s="57"/>
@@ -14491,7 +14485,7 @@
     </row>
     <row r="545" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A545" s="57" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B545" s="57"/>
       <c r="C545" s="57"/>
@@ -14502,7 +14496,7 @@
       <c r="F545" s="57"/>
       <c r="G545" s="57"/>
       <c r="H545" s="57" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="I545" s="57"/>
       <c r="J545" s="57"/>
@@ -14522,7 +14516,7 @@
     </row>
     <row r="546" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A546" s="57" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B546" s="57"/>
       <c r="C546" s="57"/>
@@ -14551,7 +14545,7 @@
     </row>
     <row r="547" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A547" s="57" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B547" s="57"/>
       <c r="C547" s="57"/>
@@ -14582,7 +14576,7 @@
     </row>
     <row r="548" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A548" s="57" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B548" s="57"/>
       <c r="C548" s="57"/>
@@ -14613,7 +14607,7 @@
     </row>
     <row r="549" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A549" s="57" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B549" s="57"/>
       <c r="C549" s="57"/>
@@ -14642,7 +14636,7 @@
     </row>
     <row r="550" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A550" s="57" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B550" s="57"/>
       <c r="C550" s="57"/>
@@ -14673,7 +14667,7 @@
     </row>
     <row r="551" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A551" s="57" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B551" s="57"/>
       <c r="C551" s="57"/>
@@ -14704,7 +14698,7 @@
     </row>
     <row r="552" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A552" s="57" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B552" s="57"/>
       <c r="C552" s="57"/>
@@ -14733,7 +14727,7 @@
     </row>
     <row r="553" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A553" s="57" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B553" s="57"/>
       <c r="C553" s="57"/>
@@ -14764,7 +14758,7 @@
     </row>
     <row r="554" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A554" s="57" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B554" s="57"/>
       <c r="C554" s="57"/>
@@ -14795,7 +14789,7 @@
     </row>
     <row r="555" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A555" s="57" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B555" s="57"/>
       <c r="C555" s="57"/>
@@ -14823,7 +14817,7 @@
     </row>
     <row r="556" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A556" s="57" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B556" s="57"/>
       <c r="C556" s="57"/>
@@ -14851,7 +14845,7 @@
     </row>
     <row r="557" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A557" s="57" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B557" s="57"/>
       <c r="C557" s="57"/>
@@ -14862,7 +14856,7 @@
       <c r="F557" s="58"/>
       <c r="G557" s="58"/>
       <c r="H557" s="57" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="I557" s="58"/>
       <c r="J557" s="57"/>
@@ -14881,7 +14875,7 @@
     </row>
     <row r="558" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A558" s="57" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B558" s="57"/>
       <c r="C558" s="57"/>
@@ -14909,7 +14903,7 @@
     </row>
     <row r="559" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A559" s="57" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B559" s="57"/>
       <c r="C559" s="57"/>
@@ -14939,7 +14933,7 @@
     </row>
     <row r="560" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A560" s="57" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B560" s="57"/>
       <c r="C560" s="57"/>
@@ -14969,7 +14963,7 @@
     </row>
     <row r="561" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A561" s="57" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B561" s="57"/>
       <c r="C561" s="57"/>
@@ -14988,7 +14982,7 @@
     </row>
     <row r="562" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A562" s="57" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B562" s="57"/>
       <c r="C562" s="57"/>
@@ -15016,7 +15010,7 @@
     </row>
     <row r="563" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A563" s="57" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B563" s="57"/>
       <c r="C563" s="57"/>
@@ -15046,7 +15040,7 @@
     </row>
     <row r="564" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A564" s="57" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B564" s="57"/>
       <c r="C564" s="57"/>
@@ -15076,7 +15070,7 @@
     </row>
     <row r="565" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A565" s="57" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B565" s="57"/>
       <c r="C565" s="57"/>
@@ -15098,7 +15092,7 @@
     </row>
     <row r="566" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A566" s="57" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B566" s="57"/>
       <c r="C566" s="57"/>
@@ -15123,7 +15117,7 @@
     </row>
     <row r="567" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A567" s="57" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B567" s="57"/>
       <c r="C567" s="57"/>
@@ -15273,12 +15267,12 @@
     </row>
     <row r="573" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A573" s="17" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B573" s="19"/>
       <c r="C573" s="19"/>
       <c r="E573" s="17" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="L573" s="17" t="s">
         <v>83</v>
@@ -15291,19 +15285,19 @@
         <v>37</v>
       </c>
       <c r="O573" s="17" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="P573" s="18"/>
     </row>
     <row r="574" spans="1:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A574" s="6" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B574" s="10"/>
       <c r="C574" s="10"/>
       <c r="D574" s="6"/>
       <c r="E574" s="6" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="F574" s="6"/>
       <c r="G574" s="6"/>
@@ -15322,18 +15316,18 @@
         <v>37</v>
       </c>
       <c r="O574" s="6" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="P574" s="18"/>
     </row>
     <row r="575" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A575" s="17" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B575" s="10"/>
       <c r="C575" s="10"/>
       <c r="D575" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="H575" s="6"/>
       <c r="L575" t="s">
@@ -16048,7 +16042,7 @@
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="C14" s="33"/>
       <c r="D14" s="33"/>

</xml_diff>

<commit_message>
Rough assumption on oat milk consumption
</commit_message>
<xml_diff>
--- a/data/default/DemandAndConversions.xlsx
+++ b/data/default/DemandAndConversions.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2736" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2738" uniqueCount="528">
   <si>
     <t>parameter</t>
   </si>
@@ -1644,6 +1644,12 @@
   </si>
   <si>
     <t>&lt;-- Adjusted to align w. stat. on net exports of milk powder after solving "cream balance"</t>
+  </si>
+  <si>
+    <t>25,000 tonnes oat okara per year 0.2L okara per L oat drink</t>
+  </si>
+  <si>
+    <t>https://www.axfoundation.se/en/projects/over-n-oat-residues</t>
   </si>
 </sst>
 </file>
@@ -1880,7 +1886,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1973,6 +1979,7 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5271,13 +5278,19 @@
       <c r="L132" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="M132" s="55">
-        <v>0</v>
+      <c r="M132" s="88">
+        <f>25000/0.2 / (M3*1000) / 365.25 * 1000</f>
+        <v>33.691964177904516</v>
       </c>
       <c r="N132" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="O132" s="15"/>
+      <c r="O132" s="15" t="s">
+        <v>526</v>
+      </c>
+      <c r="P132" t="s">
+        <v>527</v>
+      </c>
     </row>
     <row r="133" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A133" s="55" t="s">

</xml_diff>

<commit_message>
Fixed mistake in parameter name for share organic blood and offals
</commit_message>
<xml_diff>
--- a/data/default/DemandAndConversions.xlsx
+++ b/data/default/DemandAndConversions.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D0E270E-EC8B-4682-9925-EC6098E27F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E2CB8A-91DA-41FD-AF4D-C3EEFFC3B09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1275" yWindow="2910" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -10444,7 +10444,7 @@
         <v>40</v>
       </c>
       <c r="M397" s="6">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N397" t="s">
         <v>37</v>
@@ -10487,7 +10487,7 @@
         <v>42</v>
       </c>
       <c r="L399" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M399" s="12">
         <f>M395*0.6+M396*0.4</f>
@@ -10511,7 +10511,7 @@
         <v>42</v>
       </c>
       <c r="L400" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M400" s="12">
         <f>M395*0.6+M396*0.4</f>

</xml_diff>

<commit_message>
Resolve recipes just before calc. prod demand to make compound feeds visible in consumption data and fixed spelling of 'recipe'
</commit_message>
<xml_diff>
--- a/data/default/DemandAndConversions.xlsx
+++ b/data/default/DemandAndConversions.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A9F66D-371D-4C04-AC8C-CA496D4DD28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{941DAB52-6E3A-4640-A4B3-3BC4738CA820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27300" yWindow="795" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2595" yWindow="2595" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -1250,12 +1250,6 @@
     <t>f_food_ingr</t>
   </si>
   <si>
-    <t>recipie</t>
-  </si>
-  <si>
-    <t>Here recipies for foods made up of several other foods can be specified (i.e. compound foods). In the model these foods are converted to their constituent foods.</t>
-  </si>
-  <si>
     <t>Import shares are applied both for the compound food and the constituent foods, so that e.g. a compound food can be specified as 100% domestic while some</t>
   </si>
   <si>
@@ -1265,9 +1259,6 @@
     <t>of its ingredients are 100% imported. For production system shares the share of the compound food are used also for its ingredients. NOTE! Conversion factors</t>
   </si>
   <si>
-    <t>are not applicable for compound foods (i.e. all fods with the 'recipie' parameter specified).</t>
-  </si>
-  <si>
     <t>Offals</t>
   </si>
   <si>
@@ -1611,6 +1602,15 @@
   </si>
   <si>
     <t xml:space="preserve"> Artichokes + Asparagus + Chillies and peppers, green (capsicum spp. and pimenta spp.) + Sweet corn frozen + Sweet corn prepared or preserved</t>
+  </si>
+  <si>
+    <t>Here recipes for foods made up of several other foods can be specified (i.e. compound foods). In the model these foods are converted to their constituent foods.</t>
+  </si>
+  <si>
+    <t>recipe</t>
+  </si>
+  <si>
+    <t>are not applicable for compound foods (i.e. all fods with the 'recipe' parameter specified).</t>
   </si>
 </sst>
 </file>
@@ -2272,7 +2272,7 @@
         <v>6</v>
       </c>
       <c r="O3" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="P3" t="s">
         <v>7</v>
@@ -2718,7 +2718,7 @@
     </row>
     <row r="27" spans="1:19" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>98</v>
@@ -2960,12 +2960,12 @@
         <v>18</v>
       </c>
       <c r="O39" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="B40" t="s">
         <v>103</v>
@@ -2981,7 +2981,7 @@
         <v>18</v>
       </c>
       <c r="O40" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
@@ -3153,7 +3153,7 @@
     </row>
     <row r="50" spans="1:19" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>217</v>
@@ -3177,7 +3177,7 @@
         <v>18</v>
       </c>
       <c r="O50" s="11" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="S50"/>
     </row>
@@ -3219,7 +3219,7 @@
         <v>18</v>
       </c>
       <c r="O52" s="11" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
@@ -3240,7 +3240,7 @@
         <v>18</v>
       </c>
       <c r="O53" s="11" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
@@ -3261,7 +3261,7 @@
         <v>18</v>
       </c>
       <c r="O54" s="11" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.25">
@@ -3430,10 +3430,10 @@
         <v>18</v>
       </c>
       <c r="O63" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="P63" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
@@ -3454,10 +3454,10 @@
         <v>18</v>
       </c>
       <c r="O64" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="P64" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
@@ -3478,10 +3478,10 @@
         <v>18</v>
       </c>
       <c r="O65" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="P65" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
@@ -3502,18 +3502,18 @@
         <v>18</v>
       </c>
       <c r="O66" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="P66" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="B67" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="L67" t="s">
         <v>17</v>
@@ -3525,15 +3525,15 @@
         <v>18</v>
       </c>
       <c r="O67" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="B68" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="L68" t="s">
         <v>17</v>
@@ -3637,10 +3637,10 @@
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="16" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="B73" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C73" s="1"/>
       <c r="D73" s="1"/>
@@ -3663,10 +3663,10 @@
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="16" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="B74" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
@@ -3689,10 +3689,10 @@
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="16" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="B75" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C75" s="1"/>
       <c r="D75" s="1"/>
@@ -3715,10 +3715,10 @@
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="16" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="B76" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C76" s="1"/>
       <c r="D76" s="1"/>
@@ -3741,10 +3741,10 @@
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="16" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="B77" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
@@ -3767,10 +3767,10 @@
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="16" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="B78" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
@@ -3793,10 +3793,10 @@
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="16" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="B79" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C79" s="1"/>
       <c r="D79" s="1"/>
@@ -3819,10 +3819,10 @@
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="16" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="B80" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
@@ -3845,10 +3845,10 @@
     </row>
     <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="16" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="B81" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
@@ -3871,10 +3871,10 @@
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="16" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="B82" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C82" s="1"/>
       <c r="D82" s="1"/>
@@ -3897,10 +3897,10 @@
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="16" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="B83" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C83" s="1"/>
       <c r="D83" s="1"/>
@@ -3923,10 +3923,10 @@
     </row>
     <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="16" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="B84" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C84" s="1"/>
       <c r="D84" s="1"/>
@@ -3949,10 +3949,10 @@
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="16" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="B85" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C85" s="1"/>
       <c r="D85" s="1"/>
@@ -4210,7 +4210,7 @@
     </row>
     <row r="97" spans="1:19" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="B97" s="11" t="s">
         <v>336</v>
@@ -4234,13 +4234,13 @@
         <v>18</v>
       </c>
       <c r="O97" s="11" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="S97"/>
     </row>
     <row r="98" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A98" s="35" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="B98" s="36"/>
       <c r="C98" s="36"/>
@@ -4288,7 +4288,7 @@
     </row>
     <row r="100" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="B100" s="11" t="s">
         <v>340</v>
@@ -4314,7 +4314,7 @@
     </row>
     <row r="101" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="B101" s="11" t="s">
         <v>340</v>
@@ -4340,7 +4340,7 @@
     </row>
     <row r="102" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="B102" s="11" t="s">
         <v>340</v>
@@ -4364,13 +4364,13 @@
         <v>18</v>
       </c>
       <c r="O102" s="11" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="S102"/>
     </row>
     <row r="103" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="B103" s="11" t="s">
         <v>340</v>
@@ -4396,7 +4396,7 @@
     </row>
     <row r="104" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="11" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B104" s="11" t="s">
         <v>340</v>
@@ -4535,7 +4535,7 @@
     </row>
     <row r="110" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="B110" s="11" t="s">
         <v>114</v>
@@ -4550,7 +4550,7 @@
         <v>18</v>
       </c>
       <c r="O110" s="11" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="S110"/>
     </row>
@@ -4591,7 +4591,7 @@
         <v>18</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
     </row>
     <row r="113" spans="1:19" x14ac:dyDescent="0.25">
@@ -4747,7 +4747,7 @@
     </row>
     <row r="121" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B121" s="11" t="s">
         <v>25</v>
@@ -4762,7 +4762,7 @@
       <c r="J121" s="38"/>
       <c r="K121" s="38"/>
       <c r="L121" s="11" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="M121" s="11">
         <v>31.9</v>
@@ -4814,10 +4814,10 @@
     </row>
     <row r="124" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A124" s="16" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="B124" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C124" s="1"/>
       <c r="D124" s="1"/>
@@ -4840,10 +4840,10 @@
     </row>
     <row r="125" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A125" s="16" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="B125" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C125" s="1"/>
       <c r="D125" s="1"/>
@@ -4866,10 +4866,10 @@
     </row>
     <row r="126" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A126" s="16" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="B126" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C126" s="1"/>
       <c r="D126" s="1"/>
@@ -4892,10 +4892,10 @@
     </row>
     <row r="127" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A127" s="16" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="B127" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C127" s="1"/>
       <c r="D127" s="1"/>
@@ -4918,10 +4918,10 @@
     </row>
     <row r="128" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A128" s="16" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="B128" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C128" s="1"/>
       <c r="D128" s="1"/>
@@ -5072,10 +5072,10 @@
         <v>18</v>
       </c>
       <c r="O133" s="11" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="P133" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="134" spans="1:19" x14ac:dyDescent="0.25">
@@ -5161,7 +5161,7 @@
     </row>
     <row r="137" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="B137" s="11" t="s">
         <v>344</v>
@@ -5341,7 +5341,7 @@
     </row>
     <row r="144" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="B144" s="11" t="s">
         <v>344</v>
@@ -5544,7 +5544,7 @@
         <v>327</v>
       </c>
       <c r="O155" s="11" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
     </row>
     <row r="156" spans="1:20" x14ac:dyDescent="0.25">
@@ -5590,10 +5590,10 @@
         <v>164</v>
       </c>
       <c r="O158" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="P158" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="159" spans="1:20" x14ac:dyDescent="0.25">
@@ -5617,10 +5617,10 @@
         <v>164</v>
       </c>
       <c r="O159" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="P159" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="T159" s="6"/>
     </row>
@@ -5644,10 +5644,10 @@
         <v>164</v>
       </c>
       <c r="O160" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="P160" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="161" spans="1:20" x14ac:dyDescent="0.25">
@@ -5670,10 +5670,10 @@
         <v>164</v>
       </c>
       <c r="O161" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="P161" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="T161" s="6"/>
     </row>
@@ -5697,10 +5697,10 @@
         <v>164</v>
       </c>
       <c r="O162" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="P162" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="163" spans="1:20" x14ac:dyDescent="0.25">
@@ -5751,7 +5751,7 @@
     </row>
     <row r="165" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="B165" t="s">
         <v>98</v>
@@ -5771,7 +5771,7 @@
     </row>
     <row r="166" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="B166" t="s">
         <v>114</v>
@@ -6509,22 +6509,22 @@
     </row>
     <row r="193" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A193" s="40" t="s">
-        <v>398</v>
+        <v>515</v>
       </c>
     </row>
     <row r="194" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A194" s="40" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="195" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A195" s="40" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="196" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A196" s="40" t="s">
-        <v>402</v>
+        <v>517</v>
       </c>
     </row>
     <row r="197" spans="1:16" x14ac:dyDescent="0.25">
@@ -6535,7 +6535,7 @@
         <v>176</v>
       </c>
       <c r="L197" t="s">
-        <v>397</v>
+        <v>516</v>
       </c>
       <c r="M197">
         <v>50</v>
@@ -6544,7 +6544,7 @@
         <v>37</v>
       </c>
       <c r="O197" s="6" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="198" spans="1:16" x14ac:dyDescent="0.25">
@@ -6555,7 +6555,7 @@
         <v>113</v>
       </c>
       <c r="L198" t="s">
-        <v>397</v>
+        <v>516</v>
       </c>
       <c r="M198">
         <v>50</v>
@@ -6569,7 +6569,7 @@
     </row>
     <row r="200" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A200" s="39" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
@@ -6589,10 +6589,10 @@
     </row>
     <row r="202" spans="1:16" x14ac:dyDescent="0.25">
       <c r="L202" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="M202" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
     </row>
     <row r="204" spans="1:16" x14ac:dyDescent="0.25">
@@ -6632,7 +6632,7 @@
         <v>37</v>
       </c>
       <c r="P205" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="206" spans="1:16" x14ac:dyDescent="0.25">
@@ -6652,7 +6652,7 @@
         <v>37</v>
       </c>
       <c r="P206" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="207" spans="1:16" x14ac:dyDescent="0.25">
@@ -6673,7 +6673,7 @@
       </c>
       <c r="O207" s="6"/>
       <c r="P207" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="208" spans="1:16" x14ac:dyDescent="0.25">
@@ -6693,7 +6693,7 @@
         <v>37</v>
       </c>
       <c r="P208" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="209" spans="2:16" x14ac:dyDescent="0.25">
@@ -6713,7 +6713,7 @@
         <v>37</v>
       </c>
       <c r="P209" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="210" spans="2:16" x14ac:dyDescent="0.25">
@@ -6734,7 +6734,7 @@
       </c>
       <c r="O210" s="6"/>
       <c r="P210" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="211" spans="2:16" x14ac:dyDescent="0.25">
@@ -6754,7 +6754,7 @@
         <v>37</v>
       </c>
       <c r="P211" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="212" spans="2:16" x14ac:dyDescent="0.25">
@@ -6774,7 +6774,7 @@
         <v>37</v>
       </c>
       <c r="P212" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="213" spans="2:16" x14ac:dyDescent="0.25">
@@ -6795,7 +6795,7 @@
       </c>
       <c r="O213" s="6"/>
       <c r="P213" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="214" spans="2:16" x14ac:dyDescent="0.25">
@@ -6815,7 +6815,7 @@
         <v>37</v>
       </c>
       <c r="P214" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="215" spans="2:16" x14ac:dyDescent="0.25">
@@ -6835,7 +6835,7 @@
         <v>37</v>
       </c>
       <c r="P215" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="216" spans="2:16" x14ac:dyDescent="0.25">
@@ -6856,7 +6856,7 @@
       </c>
       <c r="O216" s="6"/>
       <c r="P216" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="217" spans="2:16" x14ac:dyDescent="0.25">
@@ -6876,10 +6876,10 @@
         <v>37</v>
       </c>
       <c r="O217" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="P217" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="218" spans="2:16" x14ac:dyDescent="0.25">
@@ -6900,7 +6900,7 @@
         <v>37</v>
       </c>
       <c r="P218" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="219" spans="2:16" x14ac:dyDescent="0.25">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="O219" s="6"/>
       <c r="P219" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="220" spans="2:16" x14ac:dyDescent="0.25">
@@ -6941,7 +6941,7 @@
         <v>37</v>
       </c>
       <c r="P220" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="221" spans="2:16" x14ac:dyDescent="0.25">
@@ -6961,7 +6961,7 @@
         <v>37</v>
       </c>
       <c r="P221" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="222" spans="2:16" x14ac:dyDescent="0.25">
@@ -6981,15 +6981,15 @@
         <v>37</v>
       </c>
       <c r="O222" s="11" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="P222" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="223" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B223" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="K223" t="s">
         <v>49</v>
@@ -7005,12 +7005,12 @@
         <v>37</v>
       </c>
       <c r="O223" s="11" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="224" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B224" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="K224" t="s">
         <v>50</v>
@@ -7029,7 +7029,7 @@
     </row>
     <row r="225" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B225" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="K225" t="s">
         <v>51</v>
@@ -7063,7 +7063,7 @@
         <v>37</v>
       </c>
       <c r="P226" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="227" spans="2:16" x14ac:dyDescent="0.25">
@@ -7083,7 +7083,7 @@
         <v>37</v>
       </c>
       <c r="P227" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="228" spans="2:16" x14ac:dyDescent="0.25">
@@ -7104,7 +7104,7 @@
       </c>
       <c r="O228" s="6"/>
       <c r="P228" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="229" spans="2:16" x14ac:dyDescent="0.25">
@@ -7124,7 +7124,7 @@
         <v>37</v>
       </c>
       <c r="P229" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="230" spans="2:16" x14ac:dyDescent="0.25">
@@ -7144,7 +7144,7 @@
         <v>37</v>
       </c>
       <c r="P230" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="231" spans="2:16" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
       </c>
       <c r="O231" s="6"/>
       <c r="P231" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="232" spans="2:16" x14ac:dyDescent="0.25">
@@ -7185,7 +7185,7 @@
         <v>37</v>
       </c>
       <c r="P232" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="233" spans="2:16" x14ac:dyDescent="0.25">
@@ -7205,7 +7205,7 @@
         <v>37</v>
       </c>
       <c r="P233" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="234" spans="2:16" x14ac:dyDescent="0.25">
@@ -7226,7 +7226,7 @@
       </c>
       <c r="O234" s="6"/>
       <c r="P234" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="235" spans="2:16" x14ac:dyDescent="0.25">
@@ -7246,7 +7246,7 @@
         <v>37</v>
       </c>
       <c r="P235" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="236" spans="2:16" x14ac:dyDescent="0.25">
@@ -7266,7 +7266,7 @@
         <v>37</v>
       </c>
       <c r="P236" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="237" spans="2:16" x14ac:dyDescent="0.25">
@@ -7287,7 +7287,7 @@
       </c>
       <c r="O237" s="6"/>
       <c r="P237" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="238" spans="2:16" x14ac:dyDescent="0.25">
@@ -7307,7 +7307,7 @@
         <v>37</v>
       </c>
       <c r="P238" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="239" spans="2:16" x14ac:dyDescent="0.25">
@@ -7327,7 +7327,7 @@
         <v>37</v>
       </c>
       <c r="P239" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="240" spans="2:16" x14ac:dyDescent="0.25">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="O240" s="6"/>
       <c r="P240" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="241" spans="1:16" x14ac:dyDescent="0.25">
@@ -7378,7 +7378,7 @@
         <v>37</v>
       </c>
       <c r="O241" s="11" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="242" spans="1:16" x14ac:dyDescent="0.25">
@@ -7464,7 +7464,7 @@
         <v>37</v>
       </c>
       <c r="O244" s="11" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="245" spans="1:16" x14ac:dyDescent="0.25">
@@ -7548,7 +7548,7 @@
       </c>
       <c r="O247" s="6"/>
       <c r="P247" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="248" spans="1:16" x14ac:dyDescent="0.25">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="O248" s="6"/>
       <c r="P248" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="249" spans="1:16" x14ac:dyDescent="0.25">
@@ -7606,7 +7606,7 @@
       </c>
       <c r="O249" s="6"/>
       <c r="P249" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="250" spans="1:16" x14ac:dyDescent="0.25">
@@ -7635,7 +7635,7 @@
       </c>
       <c r="O250" s="6"/>
       <c r="P250" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="251" spans="1:16" x14ac:dyDescent="0.25">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="O251" s="6"/>
       <c r="P251" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="252" spans="1:16" x14ac:dyDescent="0.25">
@@ -7693,12 +7693,12 @@
       </c>
       <c r="O252" s="6"/>
       <c r="P252" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="253" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B253" s="11" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C253" s="11"/>
       <c r="D253" s="11"/>
@@ -7724,7 +7724,7 @@
     </row>
     <row r="254" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B254" s="11" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C254" s="11"/>
       <c r="D254" s="11"/>
@@ -7750,7 +7750,7 @@
     </row>
     <row r="255" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B255" s="11" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C255" s="11"/>
       <c r="D255" s="11"/>
@@ -7776,7 +7776,7 @@
     </row>
     <row r="256" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B256" s="11" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C256" s="11"/>
       <c r="D256" s="11"/>
@@ -7802,7 +7802,7 @@
     </row>
     <row r="257" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B257" s="11" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C257" s="11"/>
       <c r="D257" s="11"/>
@@ -7828,7 +7828,7 @@
     </row>
     <row r="258" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B258" s="11" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C258" s="11"/>
       <c r="D258" s="11"/>
@@ -8499,7 +8499,7 @@
         <v>37</v>
       </c>
       <c r="O299" s="6" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
     </row>
     <row r="300" spans="1:16" x14ac:dyDescent="0.25">
@@ -8516,7 +8516,7 @@
         <v>37</v>
       </c>
       <c r="O300" s="6" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="301" spans="1:16" x14ac:dyDescent="0.25">
@@ -8552,7 +8552,7 @@
     </row>
     <row r="303" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A303" s="11" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="L303" t="s">
         <v>39</v>
@@ -8775,10 +8775,10 @@
         <v>37</v>
       </c>
       <c r="O316" s="11" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="P316" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="317" spans="1:16" x14ac:dyDescent="0.25">
@@ -8795,10 +8795,10 @@
         <v>37</v>
       </c>
       <c r="O317" s="11" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="P317" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="318" spans="1:16" x14ac:dyDescent="0.25">
@@ -8815,10 +8815,10 @@
         <v>37</v>
       </c>
       <c r="O318" s="11" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="P318" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="319" spans="1:16" x14ac:dyDescent="0.25">
@@ -8835,15 +8835,15 @@
         <v>37</v>
       </c>
       <c r="O319" s="11" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="P319" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="320" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="L320" t="s">
         <v>39</v>
@@ -8855,12 +8855,12 @@
         <v>37</v>
       </c>
       <c r="O320" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="321" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="L321" t="s">
         <v>39</v>
@@ -9135,7 +9135,7 @@
     </row>
     <row r="336" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A336" s="35" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="B336" s="36"/>
       <c r="C336" s="36"/>
@@ -10670,7 +10670,7 @@
     </row>
     <row r="406" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="I406" t="s">
         <v>83</v>
@@ -10689,12 +10689,12 @@
         <v>37</v>
       </c>
       <c r="O406" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="407" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="I407" t="s">
         <v>83</v>
@@ -10713,7 +10713,7 @@
         <v>37</v>
       </c>
       <c r="O407" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
     </row>
     <row r="408" spans="1:16" x14ac:dyDescent="0.25">
@@ -10893,7 +10893,7 @@
     </row>
     <row r="416" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A416" s="35" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="B416" s="36"/>
       <c r="C416" s="36"/>
@@ -11722,7 +11722,7 @@
         <v>363</v>
       </c>
       <c r="D455" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="L455" t="s">
         <v>81</v>
@@ -12279,7 +12279,7 @@
       </c>
       <c r="R484" s="48"/>
       <c r="S484" s="49" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="485" spans="1:22" x14ac:dyDescent="0.25">
@@ -12302,7 +12302,7 @@
       <c r="O485" s="5"/>
       <c r="P485" s="5"/>
       <c r="R485" s="45" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="S485" s="51">
         <v>4.2000000000000003E-2</v>
@@ -12310,7 +12310,7 @@
     </row>
     <row r="486" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A486" s="1" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="B486" s="1"/>
       <c r="C486" s="1"/>
@@ -12593,7 +12593,7 @@
         <v>37</v>
       </c>
       <c r="O493" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="P493" t="s">
         <v>88</v>
@@ -12706,7 +12706,7 @@
         <v>37</v>
       </c>
       <c r="O496" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="P496" t="s">
         <v>88</v>
@@ -12716,7 +12716,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
       <c r="T496" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
     </row>
     <row r="497" spans="1:19" x14ac:dyDescent="0.25">
@@ -12759,7 +12759,7 @@
     </row>
     <row r="498" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A498" s="38" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="B498" s="11"/>
       <c r="C498" s="11"/>
@@ -13001,7 +13001,7 @@
     </row>
     <row r="505" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A505" s="38" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B505" s="11"/>
       <c r="C505" s="11"/>
@@ -13163,10 +13163,10 @@
         <v>37</v>
       </c>
       <c r="O510" s="14" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="P510" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="511" spans="1:19" x14ac:dyDescent="0.25">
@@ -13180,7 +13180,7 @@
         <v>54</v>
       </c>
       <c r="H511" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="L511" t="s">
         <v>82</v>
@@ -13210,7 +13210,7 @@
         <v>54</v>
       </c>
       <c r="H512" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="L512" t="s">
         <v>82</v>
@@ -13240,7 +13240,7 @@
         <v>54</v>
       </c>
       <c r="H513" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="L513" t="s">
         <v>82</v>
@@ -13270,7 +13270,7 @@
         <v>54</v>
       </c>
       <c r="H514" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="L514" t="s">
         <v>82</v>
@@ -13283,10 +13283,10 @@
         <v>37</v>
       </c>
       <c r="O514" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="P514" s="42" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
     <row r="515" spans="1:16" x14ac:dyDescent="0.25">
@@ -13300,7 +13300,7 @@
         <v>54</v>
       </c>
       <c r="H515" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="L515" t="s">
         <v>82</v>
@@ -13335,10 +13335,10 @@
         <v>37</v>
       </c>
       <c r="O516" s="14" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="P516" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="517" spans="1:16" x14ac:dyDescent="0.25">
@@ -13352,7 +13352,7 @@
         <v>54</v>
       </c>
       <c r="H517" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="L517" t="s">
         <v>82</v>
@@ -13382,7 +13382,7 @@
         <v>54</v>
       </c>
       <c r="H518" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="L518" t="s">
         <v>82</v>
@@ -13412,7 +13412,7 @@
         <v>54</v>
       </c>
       <c r="H519" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="L519" t="s">
         <v>82</v>
@@ -13442,7 +13442,7 @@
         <v>54</v>
       </c>
       <c r="H520" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="L520" t="s">
         <v>82</v>
@@ -13455,10 +13455,10 @@
         <v>37</v>
       </c>
       <c r="O520" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="P520" s="42" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
     <row r="521" spans="1:16" x14ac:dyDescent="0.25">
@@ -13472,7 +13472,7 @@
         <v>54</v>
       </c>
       <c r="H521" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="L521" t="s">
         <v>82</v>
@@ -13507,10 +13507,10 @@
         <v>37</v>
       </c>
       <c r="O522" s="14" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="P522" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="523" spans="1:16" x14ac:dyDescent="0.25">
@@ -13524,7 +13524,7 @@
         <v>54</v>
       </c>
       <c r="H523" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="I523" s="16"/>
       <c r="J523" s="16"/>
@@ -13557,7 +13557,7 @@
         <v>54</v>
       </c>
       <c r="H524" s="16" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="L524" t="s">
         <v>82</v>
@@ -13587,7 +13587,7 @@
         <v>54</v>
       </c>
       <c r="H525" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="L525" t="s">
         <v>82</v>
@@ -13600,7 +13600,7 @@
         <v>37</v>
       </c>
       <c r="O525" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="P525" s="16"/>
     </row>
@@ -13615,7 +13615,7 @@
         <v>54</v>
       </c>
       <c r="H526" s="16" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="L526" t="s">
         <v>82</v>
@@ -13654,10 +13654,10 @@
         <v>37</v>
       </c>
       <c r="O527" s="14" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="P527" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="528" spans="1:16" x14ac:dyDescent="0.25">
@@ -13675,7 +13675,7 @@
         <v>54</v>
       </c>
       <c r="H528" s="16" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="L528" t="s">
         <v>82</v>
@@ -13688,10 +13688,10 @@
         <v>37</v>
       </c>
       <c r="O528" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="P528" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="529" spans="1:16" x14ac:dyDescent="0.25">
@@ -13709,7 +13709,7 @@
         <v>54</v>
       </c>
       <c r="H529" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="L529" t="s">
         <v>82</v>
@@ -13722,7 +13722,7 @@
         <v>37</v>
       </c>
       <c r="P529" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="530" spans="1:16" x14ac:dyDescent="0.25">
@@ -13740,7 +13740,7 @@
         <v>54</v>
       </c>
       <c r="H530" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="L530" t="s">
         <v>82</v>
@@ -13753,7 +13753,7 @@
         <v>37</v>
       </c>
       <c r="P530" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="531" spans="1:16" x14ac:dyDescent="0.25">
@@ -13768,10 +13768,10 @@
     </row>
     <row r="532" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A532" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="H532" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="L532" t="s">
         <v>81</v>
@@ -13785,10 +13785,10 @@
     </row>
     <row r="533" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A533" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="H533" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="L533" t="s">
         <v>81</v>
@@ -14022,7 +14022,7 @@
       <c r="B546"/>
       <c r="C546"/>
       <c r="D546" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="E546"/>
       <c r="F546"/>
@@ -14048,13 +14048,13 @@
       <c r="B547"/>
       <c r="C547"/>
       <c r="D547" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="E547"/>
       <c r="F547"/>
       <c r="G547"/>
       <c r="H547" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="I547"/>
       <c r="J547"/>
@@ -14076,7 +14076,7 @@
       <c r="B548"/>
       <c r="C548"/>
       <c r="D548" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="E548"/>
       <c r="F548"/>
@@ -14102,13 +14102,13 @@
       <c r="B549"/>
       <c r="C549"/>
       <c r="D549" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="E549"/>
       <c r="F549"/>
       <c r="G549"/>
       <c r="H549" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="I549"/>
       <c r="J549"/>
@@ -14399,7 +14399,7 @@
         <v>382</v>
       </c>
       <c r="H562" s="11" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="L562" s="11" t="s">
         <v>82</v>
@@ -14818,7 +14818,7 @@
         <v>37</v>
       </c>
       <c r="O579" s="11" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="P579" s="6"/>
     </row>
@@ -15510,7 +15510,7 @@
     </row>
     <row r="611" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A611" s="16" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="D611" s="16"/>
       <c r="L611" s="11" t="s">
@@ -15523,12 +15523,12 @@
         <v>37</v>
       </c>
       <c r="O611" s="11" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
     </row>
     <row r="612" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A612" s="16" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D612" s="16"/>
       <c r="L612" s="11" t="s">
@@ -15543,7 +15543,7 @@
     </row>
     <row r="613" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A613" s="16" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="D613" s="16"/>
       <c r="L613" s="11" t="s">
@@ -15558,7 +15558,7 @@
     </row>
     <row r="614" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A614" s="16" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="D614" s="16"/>
       <c r="L614" s="11" t="s">
@@ -15573,7 +15573,7 @@
     </row>
     <row r="615" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A615" s="16" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D615" s="16"/>
       <c r="L615" s="11" t="s">
@@ -15588,7 +15588,7 @@
     </row>
     <row r="616" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A616" s="16" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="D616" s="16"/>
       <c r="L616" s="11" t="s">
@@ -15603,7 +15603,7 @@
     </row>
     <row r="617" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A617" s="16" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="D617" s="16"/>
       <c r="L617" s="11" t="s">
@@ -15618,7 +15618,7 @@
     </row>
     <row r="618" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A618" s="16" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="D618" s="16"/>
       <c r="L618" s="11" t="s">
@@ -15633,7 +15633,7 @@
     </row>
     <row r="619" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A619" s="16" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="D619" s="16"/>
       <c r="L619" s="11" t="s">
@@ -15648,7 +15648,7 @@
     </row>
     <row r="620" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A620" s="16" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="D620" s="16"/>
       <c r="L620" s="11" t="s">
@@ -15663,7 +15663,7 @@
     </row>
     <row r="621" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A621" s="16" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="D621" s="16"/>
       <c r="L621" s="11" t="s">
@@ -15678,7 +15678,7 @@
     </row>
     <row r="622" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A622" s="16" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="D622" s="16"/>
       <c r="L622" s="11" t="s">
@@ -15693,7 +15693,7 @@
     </row>
     <row r="623" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A623" s="16" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="D623" s="16"/>
       <c r="L623" s="11" t="s">
@@ -15743,7 +15743,7 @@
     </row>
     <row r="626" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A626" s="16" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="L626" s="11" t="s">
         <v>81</v>
@@ -15757,7 +15757,7 @@
     </row>
     <row r="627" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A627" s="16" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="L627" s="11" t="s">
         <v>81</v>
@@ -15771,7 +15771,7 @@
     </row>
     <row r="628" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A628" s="16" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="L628" s="11" t="s">
         <v>81</v>
@@ -15785,7 +15785,7 @@
     </row>
     <row r="629" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A629" s="16" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="L629" s="11" t="s">
         <v>81</v>
@@ -15799,7 +15799,7 @@
     </row>
     <row r="630" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A630" s="16" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="L630" s="11" t="s">
         <v>81</v>
@@ -16121,7 +16121,7 @@
     </row>
     <row r="644" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A644" s="6" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
     </row>
   </sheetData>
@@ -16619,7 +16619,7 @@
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="C14" s="23"/>
       <c r="D14" s="23"/>

</xml_diff>